<commit_message>
Fix: Kontering in HeromaWeb (not tested)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="60">
   <si>
     <t>Name</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t>CitizensAPIVersion</t>
+  </si>
+  <si>
+    <t>BefattningsLista</t>
   </si>
 </sst>
 </file>
@@ -3030,7 +3033,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>